<commit_message>
pemindahan import -> queue
</commit_message>
<xml_diff>
--- a/resources/templates/imports/reseller-import-template.xlsx
+++ b/resources/templates/imports/reseller-import-template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/1103f4f64585d732/Documents/template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8630EEA1-B407-4B84-8547-41144DAD33F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1252BE4-969F-4FA6-BFF7-806A52504055}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{CD910885-3487-4770-B691-68481FF07D52}"/>
   </bookViews>
@@ -87,7 +87,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -110,24 +110,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -443,81 +472,77 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EC0831C9-8F41-4C05-B544-534A53E6F3A7}">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.77734375" style="3" customWidth="1"/>
-    <col min="2" max="2" width="20.88671875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="22.6640625" style="3" customWidth="1"/>
-    <col min="4" max="4" width="25.44140625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="20.77734375" style="2" customWidth="1"/>
+    <col min="2" max="2" width="20.88671875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.6640625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="25.44140625" style="2" customWidth="1"/>
     <col min="6" max="6" width="17.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="F1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="6"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>5</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F3" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="G3" s="4"/>
+      <c r="F3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F4" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>6</v>
+      <c r="F4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F5" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F6" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="F7" s="3" t="s">
+      <c r="F5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="G5" s="3" t="s">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
-    <mergeCell ref="F3:G3"/>
+    <mergeCell ref="F1:G1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>